<commit_message>
Complete Birth validation engine v1
</commit_message>
<xml_diff>
--- a/data/output/flags/flag_report.xlsx
+++ b/data/output/flags/flag_report.xlsx
@@ -4226,7 +4226,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Missing sex</t>
+          <t>Missing Sex</t>
         </is>
       </c>
       <c r="E163" t="n">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Missing nature_of_birth</t>
+          <t>Missing Nature of Birth</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E173" t="n">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -4709,7 +4709,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -4778,7 +4778,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -4801,7 +4801,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Missing birth_weight</t>
+          <t>Missing Birth Weight</t>
         </is>
       </c>
       <c r="E181" t="n">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E182" t="n">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Missing mother_age</t>
+          <t>Missing Mother Age</t>
         </is>
       </c>
       <c r="E190" t="n">

</xml_diff>